<commit_message>
new updates on files for 8/4
</commit_message>
<xml_diff>
--- a/output/mariners_report_20260804.xlsx
+++ b/output/mariners_report_20260804.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roster Moves" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trade Targets" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deadline Simulation" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -149,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -334,6 +335,7 @@
     <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -7589,4 +7591,2841 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G173"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DEADLINE ACQUISITION SIMULATOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SCENARIO SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Proj W</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Final</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="37" t="inlineStr">
+        <is>
+          <t>Baseline - no moves, no IL returns</t>
+        </is>
+      </c>
+      <c r="B4" s="46" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="C4" s="46" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="D4" s="40" t="n">
+        <v>0.503</v>
+      </c>
+      <c r="E4" s="39" t="n">
+        <v>29</v>
+      </c>
+      <c r="F4" s="39" t="inlineStr">
+        <is>
+          <t>84-78</t>
+        </is>
+      </c>
+      <c r="G4" s="38" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="37" t="inlineStr">
+        <is>
+          <t>IL Returns Only - no deadline moves</t>
+        </is>
+      </c>
+      <c r="B5" s="46" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C5" s="46" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="D5" s="40" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="E5" s="39" t="n">
+        <v>31</v>
+      </c>
+      <c r="F5" s="39" t="inlineStr">
+        <is>
+          <t>86-76</t>
+        </is>
+      </c>
+      <c r="G5" s="38" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="inlineStr">
+        <is>
+          <t>IL Returns + YES Targets (Eldridge + Bleday + Jeffers)</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="C6" s="46" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="D6" s="40" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="E6" s="39" t="n">
+        <v>32</v>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>87-75</t>
+        </is>
+      </c>
+      <c r="G6" s="38" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="inlineStr">
+        <is>
+          <t>IL Returns + YES + Pitching (+ Lee + Varland)</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="C7" s="46" t="n">
+        <v>3.64</v>
+      </c>
+      <c r="D7" s="40" t="n">
+        <v>0.594</v>
+      </c>
+      <c r="E7" s="39" t="n">
+        <v>33</v>
+      </c>
+      <c r="F7" s="39" t="inlineStr">
+        <is>
+          <t>88-74</t>
+        </is>
+      </c>
+      <c r="G7" s="38" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>IL Returns + MAYBE (Dingler + Vargas + Contreras)</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="C8" s="46" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="D8" s="40" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="E8" s="39" t="n">
+        <v>32</v>
+      </c>
+      <c r="F8" s="39" t="inlineStr">
+        <is>
+          <t>87-75</t>
+        </is>
+      </c>
+      <c r="G8" s="38" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>Best Case - All IL + YES + Pitching</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="n">
+        <v>4.48</v>
+      </c>
+      <c r="C9" s="46" t="n">
+        <v>3.57</v>
+      </c>
+      <c r="D9" s="40" t="n">
+        <v>0.603</v>
+      </c>
+      <c r="E9" s="39" t="n">
+        <v>33</v>
+      </c>
+      <c r="F9" s="39" t="inlineStr">
+        <is>
+          <t>88-74</t>
+        </is>
+      </c>
+      <c r="G9" s="38" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>Worst Case - No moves, Julio slow return</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="C10" s="46" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="D10" s="40" t="n">
+        <v>0.525</v>
+      </c>
+      <c r="E10" s="39" t="n">
+        <v>30</v>
+      </c>
+      <c r="F10" s="39" t="inlineStr">
+        <is>
+          <t>85-77</t>
+        </is>
+      </c>
+      <c r="G10" s="38" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>Optimistic IL - Everyone Returns Early</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="C11" s="46" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="D11" s="40" t="n">
+        <v>0.546</v>
+      </c>
+      <c r="E11" s="39" t="n">
+        <v>31</v>
+      </c>
+      <c r="F11" s="39" t="inlineStr">
+        <is>
+          <t>86-76</t>
+        </is>
+      </c>
+      <c r="G11" s="38" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>Pessimistic IL - Setbacks, Late Returns</t>
+        </is>
+      </c>
+      <c r="B12" s="46" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="C12" s="46" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="D12" s="40" t="n">
+        <v>0.5629999999999999</v>
+      </c>
+      <c r="E12" s="39" t="n">
+        <v>31</v>
+      </c>
+      <c r="F12" s="39" t="inlineStr">
+        <is>
+          <t>86-76</t>
+        </is>
+      </c>
+      <c r="G12" s="38" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>BASELINE - NO MOVES, NO IL RETURNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="B15" s="62" t="n">
+        <v>4.02</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B16" s="62" t="n">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B17" s="62" t="n">
+        <v>0.503</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B18" s="62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>Final W-L</t>
+        </is>
+      </c>
+      <c r="B19" s="62" t="inlineStr">
+        <is>
+          <t>84-78</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B20" s="62" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B21" s="62" t="inlineStr">
+        <is>
+          <t>+1 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B22" s="62" t="inlineStr">
+        <is>
+          <t>+5 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>IL RETURNS ONLY - NO DEADLINE MOVES</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="B25" s="62" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B26" s="62" t="n">
+        <v>3.81</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B27" s="62" t="n">
+        <v>0.545</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B28" s="62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>Final W-L</t>
+        </is>
+      </c>
+      <c r="B29" s="62" t="inlineStr">
+        <is>
+          <t>86-76</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B30" s="62" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B31" s="62" t="inlineStr">
+        <is>
+          <t>+3 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B32" s="62" t="inlineStr">
+        <is>
+          <t>+7 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Brendan Donovan</t>
+        </is>
+      </c>
+      <c r="B34" s="39" t="inlineStr">
+        <is>
+          <t>+0.140</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" s="22" t="inlineStr">
+        <is>
+          <t>.839 OPS when healthy - est Jul 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Will Wilson</t>
+        </is>
+      </c>
+      <c r="B35" s="39" t="inlineStr">
+        <is>
+          <t>+0.040</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="22" t="inlineStr">
+        <is>
+          <t>Bench depth - est Jul 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>-0.100</t>
+        </is>
+      </c>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t>0.54 ERA closer - est Jul 20 from 15-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C37" s="39" t="inlineStr">
+        <is>
+          <t>-0.050</t>
+        </is>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth - est Aug 3 from 60-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C38" s="39" t="inlineStr">
+        <is>
+          <t>-0.032</t>
+        </is>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>60-day IL - return date uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>Luck correction</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>Luck -2.0 - ~1 free wins</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>IL RETURNS + YES TARGETS (ELDRIDGE + BLEDAY + JEFFERS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="B42" s="62" t="n">
+        <v>4.48</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B43" s="62" t="n">
+        <v>3.81</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B44" s="62" t="n">
+        <v>0.574</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="21" t="inlineStr">
+        <is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B45" s="62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="21" t="inlineStr">
+        <is>
+          <t>Final W-L</t>
+        </is>
+      </c>
+      <c r="B46" s="62" t="inlineStr">
+        <is>
+          <t>87-75</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B47" s="62" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B48" s="62" t="inlineStr">
+        <is>
+          <t>+4 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="21" t="inlineStr">
+        <is>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B49" s="62" t="inlineStr">
+        <is>
+          <t>+8 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Brendan Donovan</t>
+        </is>
+      </c>
+      <c r="B51" s="39" t="inlineStr">
+        <is>
+          <t>+0.140</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D51" s="22" t="inlineStr">
+        <is>
+          <t>.839 OPS when healthy - est Jul 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Will Wilson</t>
+        </is>
+      </c>
+      <c r="B52" s="39" t="inlineStr">
+        <is>
+          <t>+0.040</t>
+        </is>
+      </c>
+      <c r="C52" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="22" t="inlineStr">
+        <is>
+          <t>Bench depth - est Jul 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C53" s="39" t="inlineStr">
+        <is>
+          <t>-0.100</t>
+        </is>
+      </c>
+      <c r="D53" s="22" t="inlineStr">
+        <is>
+          <t>0.54 ERA closer - est Jul 20 from 15-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C54" s="39" t="inlineStr">
+        <is>
+          <t>-0.050</t>
+        </is>
+      </c>
+      <c r="D54" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth - est Aug 3 from 60-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C55" s="39" t="inlineStr">
+        <is>
+          <t>-0.032</t>
+        </is>
+      </c>
+      <c r="D55" s="22" t="inlineStr">
+        <is>
+          <t>60-day IL - return date uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Dominic Smith</t>
+        </is>
+      </c>
+      <c r="B56" s="39" t="inlineStr">
+        <is>
+          <t>+0.100</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="22" t="inlineStr">
+        <is>
+          <t>Cheap ATL DH, squeezed by Acuna/Murphy returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: JJ Bleday</t>
+        </is>
+      </c>
+      <c r="B57" s="39" t="inlineStr">
+        <is>
+          <t>+0.100</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="22" t="inlineStr">
+        <is>
+          <t>OF depth, .399 xwOBA, 14 HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Ryan Jeffers</t>
+        </is>
+      </c>
+      <c r="B58" s="39" t="inlineStr">
+        <is>
+          <t>+0.080</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="22" t="inlineStr">
+        <is>
+          <t>.949 OPS, insurance/DH flexibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="21" t="inlineStr">
+        <is>
+          <t>Luck correction</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D59" s="22" t="inlineStr">
+        <is>
+          <t>Luck -2.0 - ~1 free wins</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>IL RETURNS + YES + PITCHING (+ LEE + VARLAND)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="21" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="B62" s="62" t="n">
+        <v>4.48</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="21" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B63" s="62" t="n">
+        <v>3.64</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="21" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B64" s="62" t="n">
+        <v>0.594</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="21" t="inlineStr">
+        <is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B65" s="62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="21" t="inlineStr">
+        <is>
+          <t>Final W-L</t>
+        </is>
+      </c>
+      <c r="B66" s="62" t="inlineStr">
+        <is>
+          <t>88-74</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B67" s="62" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B68" s="62" t="inlineStr">
+        <is>
+          <t>+5 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="21" t="inlineStr">
+        <is>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B69" s="62" t="inlineStr">
+        <is>
+          <t>+9 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Brendan Donovan</t>
+        </is>
+      </c>
+      <c r="B71" s="39" t="inlineStr">
+        <is>
+          <t>+0.140</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D71" s="22" t="inlineStr">
+        <is>
+          <t>.839 OPS when healthy - est Jul 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Will Wilson</t>
+        </is>
+      </c>
+      <c r="B72" s="39" t="inlineStr">
+        <is>
+          <t>+0.040</t>
+        </is>
+      </c>
+      <c r="C72" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D72" s="22" t="inlineStr">
+        <is>
+          <t>Bench depth - est Jul 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C73" s="39" t="inlineStr">
+        <is>
+          <t>-0.100</t>
+        </is>
+      </c>
+      <c r="D73" s="22" t="inlineStr">
+        <is>
+          <t>0.54 ERA closer - est Jul 20 from 15-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C74" s="39" t="inlineStr">
+        <is>
+          <t>-0.050</t>
+        </is>
+      </c>
+      <c r="D74" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth - est Aug 3 from 60-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C75" s="39" t="inlineStr">
+        <is>
+          <t>-0.032</t>
+        </is>
+      </c>
+      <c r="D75" s="22" t="inlineStr">
+        <is>
+          <t>60-day IL - return date uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Dominic Smith</t>
+        </is>
+      </c>
+      <c r="B76" s="39" t="inlineStr">
+        <is>
+          <t>+0.100</t>
+        </is>
+      </c>
+      <c r="C76" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D76" s="22" t="inlineStr">
+        <is>
+          <t>Cheap ATL DH, squeezed by Acuna/Murphy returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: JJ Bleday</t>
+        </is>
+      </c>
+      <c r="B77" s="39" t="inlineStr">
+        <is>
+          <t>+0.100</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D77" s="22" t="inlineStr">
+        <is>
+          <t>OF depth, .399 xwOBA, 14 HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Ryan Jeffers</t>
+        </is>
+      </c>
+      <c r="B78" s="39" t="inlineStr">
+        <is>
+          <t>+0.080</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D78" s="22" t="inlineStr">
+        <is>
+          <t>.949 OPS, insurance/DH flexibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Dylan Lee</t>
+        </is>
+      </c>
+      <c r="B79" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C79" s="39" t="inlineStr">
+        <is>
+          <t>-0.090</t>
+        </is>
+      </c>
+      <c r="D79" s="22" t="inlineStr">
+        <is>
+          <t>Elite .209 xwOBA, 1.52 ERA</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Louis Varland</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C80" s="39" t="inlineStr">
+        <is>
+          <t>-0.080</t>
+        </is>
+      </c>
+      <c r="D80" s="22" t="inlineStr">
+        <is>
+          <t>Elite .216 xwOBA, 0.94 ERA</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="21" t="inlineStr">
+        <is>
+          <t>Luck correction</t>
+        </is>
+      </c>
+      <c r="B81" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>Luck -2.0 - ~1 free wins</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>IL RETURNS + MAYBE (DINGLER + VARGAS + CONTRERAS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="21" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="B84" s="62" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="21" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B85" s="62" t="n">
+        <v>3.81</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="21" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B86" s="62" t="n">
+        <v>0.575</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="21" t="inlineStr">
+        <is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B87" s="62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="21" t="inlineStr">
+        <is>
+          <t>Final W-L</t>
+        </is>
+      </c>
+      <c r="B88" s="62" t="inlineStr">
+        <is>
+          <t>87-75</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B89" s="62" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B90" s="62" t="inlineStr">
+        <is>
+          <t>+4 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="21" t="inlineStr">
+        <is>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B91" s="62" t="inlineStr">
+        <is>
+          <t>+8 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Brendan Donovan</t>
+        </is>
+      </c>
+      <c r="B93" s="39" t="inlineStr">
+        <is>
+          <t>+0.140</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D93" s="22" t="inlineStr">
+        <is>
+          <t>.839 OPS when healthy - est Jul 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Will Wilson</t>
+        </is>
+      </c>
+      <c r="B94" s="39" t="inlineStr">
+        <is>
+          <t>+0.040</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D94" s="22" t="inlineStr">
+        <is>
+          <t>Bench depth - est Jul 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B95" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C95" s="39" t="inlineStr">
+        <is>
+          <t>-0.100</t>
+        </is>
+      </c>
+      <c r="D95" s="22" t="inlineStr">
+        <is>
+          <t>0.54 ERA closer - est Jul 20 from 15-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B96" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C96" s="39" t="inlineStr">
+        <is>
+          <t>-0.050</t>
+        </is>
+      </c>
+      <c r="D96" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth - est Aug 3 from 60-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B97" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C97" s="39" t="inlineStr">
+        <is>
+          <t>-0.032</t>
+        </is>
+      </c>
+      <c r="D97" s="22" t="inlineStr">
+        <is>
+          <t>60-day IL - return date uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Dillon Dingler</t>
+        </is>
+      </c>
+      <c r="B98" s="39" t="inlineStr">
+        <is>
+          <t>+0.110</t>
+        </is>
+      </c>
+      <c r="C98" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D98" s="22" t="inlineStr">
+        <is>
+          <t>Tigers seller, .409 xwOBA, 19 HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Miguel Vargas</t>
+        </is>
+      </c>
+      <c r="B99" s="39" t="inlineStr">
+        <is>
+          <t>+0.090</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D99" s="22" t="inlineStr">
+        <is>
+          <t>Versatile, .397 xwOBA, 20 HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Carlos Cortes</t>
+        </is>
+      </c>
+      <c r="B100" s="39" t="inlineStr">
+        <is>
+          <t>+0.090</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D100" s="22" t="inlineStr">
+        <is>
+          <t>A's breakout OF, minor-league find, no long-term commitment</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="21" t="inlineStr">
+        <is>
+          <t>Luck correction</t>
+        </is>
+      </c>
+      <c r="B101" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D101" s="22" t="inlineStr">
+        <is>
+          <t>Luck -2.0 - ~1 free wins</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="20" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>BEST CASE - ALL IL + YES + PITCHING</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="21" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="B104" s="62" t="n">
+        <v>4.48</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="21" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B105" s="62" t="n">
+        <v>3.57</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="21" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B106" s="62" t="n">
+        <v>0.603</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="21" t="inlineStr">
+        <is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B107" s="62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="21" t="inlineStr">
+        <is>
+          <t>Final W-L</t>
+        </is>
+      </c>
+      <c r="B108" s="62" t="inlineStr">
+        <is>
+          <t>88-74</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B109" s="62" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B110" s="62" t="inlineStr">
+        <is>
+          <t>+5 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="21" t="inlineStr">
+        <is>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B111" s="62" t="inlineStr">
+        <is>
+          <t>+9 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B112" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D112" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Brendan Donovan</t>
+        </is>
+      </c>
+      <c r="B113" s="39" t="inlineStr">
+        <is>
+          <t>+0.140</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D113" s="22" t="inlineStr">
+        <is>
+          <t>.839 OPS when healthy - est Jul 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Will Wilson</t>
+        </is>
+      </c>
+      <c r="B114" s="39" t="inlineStr">
+        <is>
+          <t>+0.040</t>
+        </is>
+      </c>
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D114" s="22" t="inlineStr">
+        <is>
+          <t>Bench depth - est Jul 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B115" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C115" s="39" t="inlineStr">
+        <is>
+          <t>-0.100</t>
+        </is>
+      </c>
+      <c r="D115" s="22" t="inlineStr">
+        <is>
+          <t>0.54 ERA closer - est Jul 20 from 15-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B116" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C116" s="39" t="inlineStr">
+        <is>
+          <t>-0.050</t>
+        </is>
+      </c>
+      <c r="D116" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth - est Aug 3 from 60-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B117" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C117" s="39" t="inlineStr">
+        <is>
+          <t>-0.032</t>
+        </is>
+      </c>
+      <c r="D117" s="22" t="inlineStr">
+        <is>
+          <t>60-day IL - return date uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Dominic Smith</t>
+        </is>
+      </c>
+      <c r="B118" s="39" t="inlineStr">
+        <is>
+          <t>+0.100</t>
+        </is>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D118" s="22" t="inlineStr">
+        <is>
+          <t>Cheap ATL DH, squeezed by Acuna/Murphy returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: JJ Bleday</t>
+        </is>
+      </c>
+      <c r="B119" s="39" t="inlineStr">
+        <is>
+          <t>+0.100</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D119" s="22" t="inlineStr">
+        <is>
+          <t>OF depth, .399 xwOBA, 14 HR</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Ryan Jeffers</t>
+        </is>
+      </c>
+      <c r="B120" s="39" t="inlineStr">
+        <is>
+          <t>+0.080</t>
+        </is>
+      </c>
+      <c r="C120" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D120" s="22" t="inlineStr">
+        <is>
+          <t>.949 OPS, insurance/DH flexibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Dylan Lee</t>
+        </is>
+      </c>
+      <c r="B121" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C121" s="39" t="inlineStr">
+        <is>
+          <t>-0.090</t>
+        </is>
+      </c>
+      <c r="D121" s="22" t="inlineStr">
+        <is>
+          <t>Elite .209 xwOBA, 1.52 ERA</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Louis Varland</t>
+        </is>
+      </c>
+      <c r="B122" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C122" s="39" t="inlineStr">
+        <is>
+          <t>-0.080</t>
+        </is>
+      </c>
+      <c r="D122" s="22" t="inlineStr">
+        <is>
+          <t>Elite .216 xwOBA, 0.94 ERA</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Raisel Iglesias</t>
+        </is>
+      </c>
+      <c r="B123" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C123" s="39" t="inlineStr">
+        <is>
+          <t>-0.070</t>
+        </is>
+      </c>
+      <c r="D123" s="22" t="inlineStr">
+        <is>
+          <t>Veteran closer/setup, 2.30 ERA</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="21" t="inlineStr">
+        <is>
+          <t>Luck correction</t>
+        </is>
+      </c>
+      <c r="B124" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C124" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D124" s="22" t="inlineStr">
+        <is>
+          <t>Luck -2.0 - ~1 free wins</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="20" customHeight="1">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>WORST CASE - NO MOVES, JULIO SLOW RETURN</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="21" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="B127" s="62" t="n">
+        <v>4.02</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="21" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B128" s="62" t="n">
+        <v>3.81</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="21" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B129" s="62" t="n">
+        <v>0.525</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="21" t="inlineStr">
+        <is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B130" s="62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="21" t="inlineStr">
+        <is>
+          <t>Final W-L</t>
+        </is>
+      </c>
+      <c r="B131" s="62" t="inlineStr">
+        <is>
+          <t>85-77</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B132" s="62" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B133" s="62" t="inlineStr">
+        <is>
+          <t>+2 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="21" t="inlineStr">
+        <is>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B134" s="62" t="inlineStr">
+        <is>
+          <t>+6 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B136" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C136" s="39" t="inlineStr">
+        <is>
+          <t>-0.100</t>
+        </is>
+      </c>
+      <c r="D136" s="22" t="inlineStr">
+        <is>
+          <t>0.54 ERA closer - est Jul 20 from 15-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B137" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C137" s="39" t="inlineStr">
+        <is>
+          <t>-0.050</t>
+        </is>
+      </c>
+      <c r="D137" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth - est Aug 3 from 60-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B138" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C138" s="39" t="inlineStr">
+        <is>
+          <t>-0.032</t>
+        </is>
+      </c>
+      <c r="D138" s="22" t="inlineStr">
+        <is>
+          <t>60-day IL - return date uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="20" customHeight="1">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>OPTIMISTIC IL - EVERYONE RETURNS EARLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="21" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="B141" s="62" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="21" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B142" s="62" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="21" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B143" s="62" t="n">
+        <v>0.546</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="21" t="inlineStr">
+        <is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B144" s="62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="21" t="inlineStr">
+        <is>
+          <t>Final W-L</t>
+        </is>
+      </c>
+      <c r="B145" s="62" t="inlineStr">
+        <is>
+          <t>86-76</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B146" s="62" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B147" s="62" t="inlineStr">
+        <is>
+          <t>+3 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="21" t="inlineStr">
+        <is>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B148" s="62" t="inlineStr">
+        <is>
+          <t>+7 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Brendan Donovan</t>
+        </is>
+      </c>
+      <c r="B150" s="39" t="inlineStr">
+        <is>
+          <t>+0.140</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D150" s="22" t="inlineStr">
+        <is>
+          <t>.839 OPS when healthy - est Jul 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Will Wilson</t>
+        </is>
+      </c>
+      <c r="B151" s="39" t="inlineStr">
+        <is>
+          <t>+0.040</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D151" s="22" t="inlineStr">
+        <is>
+          <t>Bench depth - est Jul 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B152" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C152" s="39" t="inlineStr">
+        <is>
+          <t>-0.100</t>
+        </is>
+      </c>
+      <c r="D152" s="22" t="inlineStr">
+        <is>
+          <t>0.54 ERA closer - est Jul 20 from 15-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B153" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C153" s="39" t="inlineStr">
+        <is>
+          <t>-0.050</t>
+        </is>
+      </c>
+      <c r="D153" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth - est Aug 3 from 60-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B154" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C154" s="39" t="inlineStr">
+        <is>
+          <t>-0.040</t>
+        </is>
+      </c>
+      <c r="D154" s="22" t="inlineStr">
+        <is>
+          <t>60-day IL - return date uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="21" t="inlineStr">
+        <is>
+          <t>Luck correction</t>
+        </is>
+      </c>
+      <c r="B155" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D155" s="22" t="inlineStr">
+        <is>
+          <t>Luck -2.0 - ~1 free wins</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="20" customHeight="1">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>PESSIMISTIC IL - SETBACKS, LATE RETURNS</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="21" t="inlineStr">
+        <is>
+          <t>RS/G</t>
+        </is>
+      </c>
+      <c r="B158" s="62" t="n">
+        <v>4.3</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="21" t="inlineStr">
+        <is>
+          <t>RA/G</t>
+        </is>
+      </c>
+      <c r="B159" s="62" t="n">
+        <v>3.74</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="21" t="inlineStr">
+        <is>
+          <t>Win%</t>
+        </is>
+      </c>
+      <c r="B160" s="62" t="n">
+        <v>0.5629999999999999</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="21" t="inlineStr">
+        <is>
+          <t>Luck wins</t>
+        </is>
+      </c>
+      <c r="B161" s="62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="21" t="inlineStr">
+        <is>
+          <t>Final W-L</t>
+        </is>
+      </c>
+      <c r="B162" s="62" t="inlineStr">
+        <is>
+          <t>86-76</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="21" t="inlineStr">
+        <is>
+          <t>Playoff</t>
+        </is>
+      </c>
+      <c r="B163" s="62" t="inlineStr">
+        <is>
+          <t>Division winner</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="21" t="inlineStr">
+        <is>
+          <t>vs TEX</t>
+        </is>
+      </c>
+      <c r="B164" s="62" t="inlineStr">
+        <is>
+          <t>+3 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="21" t="inlineStr">
+        <is>
+          <t>vs HOU</t>
+        </is>
+      </c>
+      <c r="B165" s="62" t="inlineStr">
+        <is>
+          <t>+7 games</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>Factor</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>RS/G impact</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>RA/G impact</t>
+        </is>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Brendan Donovan</t>
+        </is>
+      </c>
+      <c r="B167" s="39" t="inlineStr">
+        <is>
+          <t>+0.140</t>
+        </is>
+      </c>
+      <c r="C167" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D167" s="22" t="inlineStr">
+        <is>
+          <t>.839 OPS when healthy - est Jul 17</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Will Wilson</t>
+        </is>
+      </c>
+      <c r="B168" s="39" t="inlineStr">
+        <is>
+          <t>+0.040</t>
+        </is>
+      </c>
+      <c r="C168" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D168" s="22" t="inlineStr">
+        <is>
+          <t>Bench depth - est Jul 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Matt Brash</t>
+        </is>
+      </c>
+      <c r="B169" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C169" s="39" t="inlineStr">
+        <is>
+          <t>-0.100</t>
+        </is>
+      </c>
+      <c r="D169" s="22" t="inlineStr">
+        <is>
+          <t>0.54 ERA closer - est Jul 20 from 15-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Carlos Vargas</t>
+        </is>
+      </c>
+      <c r="B170" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C170" s="39" t="inlineStr">
+        <is>
+          <t>-0.038</t>
+        </is>
+      </c>
+      <c r="D170" s="22" t="inlineStr">
+        <is>
+          <t>Bullpen depth - est Aug 3 from 60-day IL</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="21" t="inlineStr">
+        <is>
+          <t>IL return: Cooper Criswell</t>
+        </is>
+      </c>
+      <c r="B171" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C171" s="39" t="inlineStr">
+        <is>
+          <t>-0.020</t>
+        </is>
+      </c>
+      <c r="D171" s="22" t="inlineStr">
+        <is>
+          <t>60-day IL - return date uncertain</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Dominic Smith</t>
+        </is>
+      </c>
+      <c r="B172" s="39" t="inlineStr">
+        <is>
+          <t>+0.100</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D172" s="22" t="inlineStr">
+        <is>
+          <t>Cheap ATL DH, squeezed by Acuna/Murphy returns</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="21" t="inlineStr">
+        <is>
+          <t>Acquired: Dylan Lee</t>
+        </is>
+      </c>
+      <c r="B173" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C173" s="39" t="inlineStr">
+        <is>
+          <t>-0.090</t>
+        </is>
+      </c>
+      <c r="D173" s="22" t="inlineStr">
+        <is>
+          <t>Elite .209 xwOBA, 1.52 ERA</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="83">
+    <mergeCell ref="B111:G111"/>
+    <mergeCell ref="B145:G145"/>
+    <mergeCell ref="A126:G126"/>
+    <mergeCell ref="A140:G140"/>
+    <mergeCell ref="B88:G88"/>
+    <mergeCell ref="B147:G147"/>
+    <mergeCell ref="B162:G162"/>
+    <mergeCell ref="B146:G146"/>
+    <mergeCell ref="B65:G65"/>
+    <mergeCell ref="B68:G68"/>
+    <mergeCell ref="A103:G103"/>
+    <mergeCell ref="B45:G45"/>
+    <mergeCell ref="B110:G110"/>
+    <mergeCell ref="B109:G109"/>
+    <mergeCell ref="B165:G165"/>
+    <mergeCell ref="B47:G47"/>
+    <mergeCell ref="B141:G141"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="B86:G86"/>
+    <mergeCell ref="B87:G87"/>
+    <mergeCell ref="B128:G128"/>
+    <mergeCell ref="A83:G83"/>
+    <mergeCell ref="B49:G49"/>
+    <mergeCell ref="A157:G157"/>
+    <mergeCell ref="B64:G64"/>
+    <mergeCell ref="B104:G104"/>
+    <mergeCell ref="B164:G164"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="B63:G63"/>
+    <mergeCell ref="B161:G161"/>
+    <mergeCell ref="B106:G106"/>
+    <mergeCell ref="B163:G163"/>
+    <mergeCell ref="B91:G91"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="B66:G66"/>
+    <mergeCell ref="B131:G131"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B130:G130"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="B67:G67"/>
+    <mergeCell ref="B132:G132"/>
+    <mergeCell ref="B29:G29"/>
+    <mergeCell ref="B69:G69"/>
+    <mergeCell ref="B84:G84"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="B127:G127"/>
+    <mergeCell ref="B158:G158"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B142:G142"/>
+    <mergeCell ref="B89:G89"/>
+    <mergeCell ref="B160:G160"/>
+    <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B144:G144"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="B129:G129"/>
+    <mergeCell ref="B134:G134"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B90:G90"/>
+    <mergeCell ref="B105:G105"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B43:G43"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="B107:G107"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B148:G148"/>
+    <mergeCell ref="B44:G44"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="B108:G108"/>
+    <mergeCell ref="B143:G143"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="A61:G61"/>
+    <mergeCell ref="B133:G133"/>
+    <mergeCell ref="B85:G85"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="B62:G62"/>
+    <mergeCell ref="B46:G46"/>
+    <mergeCell ref="B159:G159"/>
+    <mergeCell ref="B48:G48"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>